<commit_message>
evidence: accept T05 PAD candidate
</commit_message>
<xml_diff>
--- a/catalog/evidence/normal-chat-t05-final.xlsx
+++ b/catalog/evidence/normal-chat-t05-final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuuki\ai-prompts\catalog\evidence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A56E4A9D-BE7E-4D56-B621-0A6FB0AEA562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E844A05-DA4B-4B8C-A424-44519B81A4CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F6C7D14D-0971-4AB2-8FFC-8F2855D3F312}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F6C7D14D-0971-4AB2-8FFC-8F2855D3F312}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -429,14 +429,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4299051A-B3B6-48D5-B84C-9AE3FEBBFD34}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" t="s">
         <v>1</v>
       </c>

</xml_diff>